<commit_message>
Fix second student audit gaps in assessment and recovery
</commit_message>
<xml_diff>
--- a/assets/lessons/excel-formula-fluency/sprint/datasets/L10-A4.xlsx
+++ b/assets/lessons/excel-formula-fluency/sprint/datasets/L10-A4.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answers" sheetId="1" r:id="R29964a7fd19948db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rc0c51fee46fa4a63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="3" r:id="R75b7303b76f3457d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Months" sheetId="4" r:id="R7c9546cc312a4452"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="5" r:id="Rd5fbfae56be54b32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionary" sheetId="6" r:id="R096855c634c34d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answers" sheetId="1" r:id="R03c56fd88ce34936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R3595a9a07c0648f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="3" r:id="Rc0ae405c1d264c65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Months" sheetId="4" r:id="Rdf22cb85b2264d4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="5" r:id="R9b28177a56d44e83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionary" sheetId="6" r:id="Racbc7faa35114556"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2546,7 +2546,7 @@
         <x:v>How to submit</x:v>
       </x:c>
       <x:c r="B3" s="23" t="str">
-        <x:v>Solve in current Microsoft 365 Excel. Answers cells are intentionally empty. Any equivalent Excel formula is accepted. Paste each requested output with its formula into the lesson. Preserve leading-zero identifiers as text. All four required tasks must pass before model solutions unlock.</x:v>
+        <x:v>Solve in current Microsoft 365 Excel. Answers cells are intentionally empty. Any equivalent formula is accepted. Submit each complete output with its formula. Preserve leading-zero identifiers as text. All four required tasks unlock models. Formula examples use commas; use semicolon argument separators if your locale requires them. Keep spill ranges empty and enter their anchor formulas outside Excel Table bodies.</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -2616,7 +2616,7 @@
         <x:v>Bonus: Answers!B23</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Review COUNTIFS: count raw lines with returns strictly greater than sold units.</x:v>
+        <x:v>Review SUMPRODUCT: count raw lines with returns strictly greater than sold units by comparing the two quantities within each row.</x:v>
       </x:c>
       <x:c r="C8" s="2"/>
       <x:c r="D8" s="2"/>
@@ -7128,7 +7128,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57249613935f4758"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ad748e75ef14e95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9163,7 +9163,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ff98c778afd43a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9f4eaf0c6b8404d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11202,7 +11202,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40a98748b57b49f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa2adfae0d5d4952"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>